<commit_message>
exp strat eval taxonomy test2
</commit_message>
<xml_diff>
--- a/results/reliability_eval/unified_scores_table_08-30-1.xlsx
+++ b/results/reliability_eval/unified_scores_table_08-30-1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -513,7 +513,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>P101</t>
+          <t>toy-qa-dataset</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -533,25 +533,25 @@
         <v>0.1</v>
       </c>
       <c r="G2" t="n">
-        <v>0.11</v>
+        <v>0.7619047619047619</v>
       </c>
       <c r="H2" t="n">
-        <v>0.2645556690500511</v>
+        <v>0.975</v>
       </c>
       <c r="I2" t="n">
-        <v>0.08126722676502246</v>
+        <v>0.9930555555555556</v>
       </c>
       <c r="J2" t="n">
-        <v>0.2645556690500511</v>
+        <v>0.975</v>
       </c>
       <c r="K2" t="n">
-        <v>0.08126722676502246</v>
+        <v>0.9930555555555556</v>
       </c>
       <c r="L2" t="n">
-        <v>0.6935648621041879</v>
+        <v>0.225</v>
       </c>
       <c r="M2" t="n">
-        <v>0.2243427942254999</v>
+        <v>0.6500599549336971</v>
       </c>
       <c r="N2" t="n">
         <v>1</v>
@@ -612,6 +612,446 @@
         <v>1</v>
       </c>
       <c r="O3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Llama-3-8B</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>toy-qa-dataset</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>fact_statement</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>beam</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.7619047619047619</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.975</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.9930555555555556</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.975</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.9930555555555556</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.225</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.6500599549336971</v>
+      </c>
+      <c r="N4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Llama-3-8B</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>toy-qa-dataset</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>fact_statement</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>beam</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>10</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.7619047619047619</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.975</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.9930555555555556</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.975</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.9930555555555556</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.225</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.6500599549336971</v>
+      </c>
+      <c r="N5" t="n">
+        <v>1</v>
+      </c>
+      <c r="O5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Llama-3-8B</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>toy-qa-dataset</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>fact_statement</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>beam</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>10</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.7619047619047619</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.975</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.9930555555555556</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.975</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.9930555555555556</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.225</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.6500599549336971</v>
+      </c>
+      <c r="N6" t="n">
+        <v>1</v>
+      </c>
+      <c r="O6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Llama-3-8B</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>toy-qa-dataset</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>fact_statement</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>beam</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.7619047619047619</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.975</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.9930555555555556</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.975</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.9930555555555556</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.225</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.6500599549336971</v>
+      </c>
+      <c r="N7" t="n">
+        <v>1</v>
+      </c>
+      <c r="O7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Llama-3-8B</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>P101</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>fact_statement</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>beam</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>10</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.3043922369765066</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.08861149780416983</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.3043922369765066</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.08861149780416983</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.5240040858018387</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.2176509266702569</v>
+      </c>
+      <c r="N8" t="n">
+        <v>1</v>
+      </c>
+      <c r="O8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Llama-3-8B</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>toy-qa-dataset</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>fact_statement</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>beam</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>10</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.7619047619047619</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.975</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.9930555555555556</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.975</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.9930555555555556</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.225</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.6500599549336971</v>
+      </c>
+      <c r="N9" t="n">
+        <v>1</v>
+      </c>
+      <c r="O9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Llama-3-8B</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>P101</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>fact_statement</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>beam</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>10</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.2645556690500511</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.08126722676502246</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.2645556690500511</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.08126722676502246</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.6935648621041879</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.2243427942254999</v>
+      </c>
+      <c r="N10" t="n">
+        <v>1</v>
+      </c>
+      <c r="O10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Llama-3-8B</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>P101</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>fact_statement</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>beam</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>10</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.4190981432360743</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.1308952862555237</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.4190981432360743</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.1308952862555237</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.4801061007957561</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0.1261792580932974</v>
+      </c>
+      <c r="N11" t="n">
+        <v>1</v>
+      </c>
+      <c r="O11" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>